<commit_message>
Document both Nimble and Jev workflows and keep workbook Read Me in sync.
Root README links main vs experiment/jev-compare; experiments README covers keys and token fields; runner docstring notes hosted Jev support.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/experiments/jev_classifier_workbook.xlsx
+++ b/experiments/jev_classifier_workbook.xlsx
@@ -629,6 +629,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="17">
       <c r="A4" s="38" t="inlineStr">
         <is>
@@ -717,7 +718,7 @@
       </c>
       <c r="B11" s="40" t="inlineStr">
         <is>
-          <t>Written by the runner: raw model JSON per record.</t>
+          <t>Written by the runner: usage_json (input/output tokens when the API returns usage) and raw_answers_json per record.</t>
         </is>
       </c>
     </row>
@@ -741,7 +742,7 @@
       </c>
       <c r="B13" s="42" t="inlineStr">
         <is>
-          <t>Written by the runner: run metadata.</t>
+          <t>Written by the runner: run metadata, including input_tokens / output_tokens / total_tokens when usage is available.</t>
         </is>
       </c>
     </row>
@@ -892,7 +893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" style="17" min="1" max="1"/>
@@ -919,7 +920,7 @@
       </c>
       <c r="B2" s="35" t="inlineStr">
         <is>
-          <t>20260930_125525</t>
+          <t>20260930_130707</t>
         </is>
       </c>
     </row>
@@ -1063,17 +1064,65 @@
       </c>
       <c r="B14" s="35" t="inlineStr">
         <is>
-          <t>/mnt/d/dev/nimble_plant/experiments/jev_classifier_workbook_20260930_125525.jsonl</t>
+          <t>/mnt/d/dev/nimble_plant/experiments/jev_classifier_workbook_20260930_130707.jsonl</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="35" t="inlineStr">
         <is>
+          <t>input_tokens</t>
+        </is>
+      </c>
+      <c r="B15" s="35" t="inlineStr">
+        <is>
+          <t>2926</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="35" t="inlineStr">
+        <is>
+          <t>output_tokens</t>
+        </is>
+      </c>
+      <c r="B16" s="35" t="inlineStr">
+        <is>
+          <t>620</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="35" t="inlineStr">
+        <is>
+          <t>total_tokens</t>
+        </is>
+      </c>
+      <c r="B17" s="35" t="inlineStr">
+        <is>
+          <t>3546</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="35" t="inlineStr">
+        <is>
+          <t>records_with_usage</t>
+        </is>
+      </c>
+      <c r="B18" s="35" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="35" t="inlineStr">
+        <is>
           <t>output_sheets</t>
         </is>
       </c>
-      <c r="B15" s="35" t="inlineStr">
+      <c r="B19" s="35" t="inlineStr">
         <is>
           <t>output_Results, output_Raw, output_Summary, output_Run_info</t>
         </is>
@@ -16061,10 +16110,10 @@
         </is>
       </c>
       <c r="I2" s="37" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="J2" s="37" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="K2" s="35" t="inlineStr">
         <is>
@@ -16072,7 +16121,7 @@
         </is>
       </c>
       <c r="L2" s="37" t="n">
-        <v>0.98</v>
+        <v>0.99</v>
       </c>
       <c r="M2" s="37" t="n">
         <v>1.99</v>
@@ -16153,7 +16202,7 @@
         <v>0.99</v>
       </c>
       <c r="M3" s="37" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="N3" s="35" t="inlineStr"/>
       <c r="O3" s="35" t="inlineStr"/>
@@ -16226,10 +16275,10 @@
         </is>
       </c>
       <c r="R4" s="37" t="n">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="S4" s="37" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="T4" s="35" t="inlineStr">
         <is>
@@ -16237,10 +16286,10 @@
         </is>
       </c>
       <c r="U4" s="37" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.84</v>
       </c>
       <c r="V4" s="37" t="n">
-        <v>1.12</v>
+        <v>1.11</v>
       </c>
       <c r="W4" s="35" t="inlineStr"/>
       <c r="X4" s="35" t="inlineStr"/>
@@ -16318,7 +16367,7 @@
         <v>0.51</v>
       </c>
       <c r="V5" s="34" t="n">
-        <v>1.23</v>
+        <v>1.25</v>
       </c>
       <c r="W5" s="32" t="inlineStr"/>
       <c r="X5" s="32" t="inlineStr"/>
@@ -16384,10 +16433,10 @@
         </is>
       </c>
       <c r="X6" s="37" t="n">
-        <v>0.89</v>
+        <v>0.84</v>
       </c>
       <c r="Y6" s="37" t="n">
-        <v>0.91</v>
+        <v>0.86</v>
       </c>
       <c r="Z6" s="35" t="inlineStr">
         <is>
@@ -16506,11 +16555,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="17" min="1" max="1"/>
-    <col width="120" customWidth="1" style="17" min="2" max="2"/>
+    <col width="40" customWidth="1" style="17" min="2" max="2"/>
+    <col width="120" customWidth="1" style="17" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -16521,6 +16571,11 @@
       </c>
       <c r="B1" s="31" t="inlineStr">
         <is>
+          <t>usage_json</t>
+        </is>
+      </c>
+      <c r="C1" s="31" t="inlineStr">
+        <is>
           <t>raw_answers_json</t>
         </is>
       </c>
@@ -16533,7 +16588,12 @@
       </c>
       <c r="B2" s="35" t="inlineStr">
         <is>
-          <t>{"pump_failure_mode": {"type": "choice", "choice": "seal", "confidence": 1.0, "probabilities": {"other": 0.0, "seal": 1.0, "bearing": 0.0, "cavitation": 0.0, "instrument": 0.0}}, "pump_containment": {"type": "noul", "noul": 0.89}, "pump_urgency": {"type": "score", "score": 1.99, "confidence": 0.98, "legend": {"0": "Can wait for the next planned window", "1": "Should be handled within days", "2": "Needs attention now"}, "probabilities": {"0": 0.0, "1": 0.01, "2": 0.99}}}</t>
+          <t>{"input_tokens": 465, "output_tokens": 92}</t>
+        </is>
+      </c>
+      <c r="C2" s="35" t="inlineStr">
+        <is>
+          <t>{"pump_failure_mode": {"type": "choice", "choice": "seal", "confidence": 1.0, "probabilities": {"bearing": 0.0, "cavitation": 0.0, "seal": 1.0, "other": 0.0, "instrument": 0.0}}, "pump_containment": {"type": "noul", "noul": 0.9}, "pump_urgency": {"type": "score", "score": 1.99, "confidence": 0.99, "legend": {"0": "Can wait for the next planned window", "1": "Should be handled within days", "2": "Needs attention now"}, "probabilities": {"0": 0.0, "1": 0.01, "2": 0.99}}}</t>
         </is>
       </c>
     </row>
@@ -16545,7 +16605,12 @@
       </c>
       <c r="B3" s="35" t="inlineStr">
         <is>
-          <t>{"pump_failure_mode": {"type": "choice", "choice": "bearing", "confidence": 1.0, "probabilities": {"other": 0.0, "bearing": 1.0, "cavitation": 0.0, "instrument": 0.0, "seal": 0.0}}, "pump_containment": {"type": "noul", "noul": 0.01}, "pump_urgency": {"type": "score", "score": 0.0, "confidence": 0.99, "legend": {"0": "Can wait for the next planned window", "1": "Should be handled within days", "2": "Needs attention now"}, "probabilities": {"0": 1.0, "1": 0.0, "2": 0.0}}}</t>
+          <t>{"input_tokens": 464, "output_tokens": 92}</t>
+        </is>
+      </c>
+      <c r="C3" s="35" t="inlineStr">
+        <is>
+          <t>{"pump_failure_mode": {"type": "choice", "choice": "bearing", "confidence": 1.0, "probabilities": {"seal": 0.0, "instrument": 0.0, "bearing": 1.0, "other": 0.0, "cavitation": 0.0}}, "pump_containment": {"type": "noul", "noul": 0.01}, "pump_urgency": {"type": "score", "score": 0.01, "confidence": 0.99, "legend": {"0": "Can wait for the next planned window", "1": "Should be handled within days", "2": "Needs attention now"}, "probabilities": {"0": 0.99, "1": 0.01, "2": 0.0}}}</t>
         </is>
       </c>
     </row>
@@ -16557,7 +16622,12 @@
       </c>
       <c r="B4" s="35" t="inlineStr">
         <is>
-          <t>{"hx_problem": {"type": "choice", "choice": "fouling", "confidence": 1.0, "probabilities": {"flow_maldistribution": 0.0, "other": 0.0, "tube_leak": 0.0, "control_valve": 0.0, "fouling": 1.0}}, "hx_crosscontam": {"type": "noul", "noul": 0.12}, "hx_impact": {"type": "score", "score": 1.12, "confidence": 0.81, "legend": {"0": "No noticeable impact", "1": "Reduced duty but operating", "2": "Major loss of duty or unit unusable"}, "probabilities": {"0": 0.0, "1": 0.87, "2": 0.13}}}</t>
+          <t>{"input_tokens": 484, "output_tokens": 102}</t>
+        </is>
+      </c>
+      <c r="C4" s="35" t="inlineStr">
+        <is>
+          <t>{"hx_problem": {"type": "choice", "choice": "fouling", "confidence": 1.0, "probabilities": {"other": 0.0, "tube_leak": 0.0, "control_valve": 0.0, "fouling": 1.0, "flow_maldistribution": 0.0}}, "hx_crosscontam": {"type": "noul", "noul": 0.13}, "hx_impact": {"type": "score", "score": 1.11, "confidence": 0.84, "legend": {"0": "No noticeable impact", "1": "Reduced duty but operating", "2": "Major loss of duty or unit unusable"}, "probabilities": {"0": 0.0, "1": 0.89, "2": 0.11}}}</t>
         </is>
       </c>
     </row>
@@ -16569,7 +16639,12 @@
       </c>
       <c r="B5" s="35" t="inlineStr">
         <is>
-          <t>{"hx_problem": {"type": "choice", "choice": "tube_leak", "confidence": 1.0, "probabilities": {"other": 0.0, "fouling": 0.0, "flow_maldistribution": 0.0, "control_valve": 0.0, "tube_leak": 1.0}}, "hx_crosscontam": {"type": "noul", "noul": 0.9}, "hx_impact": {"type": "score", "score": 1.23, "confidence": 0.51, "legend": {"0": "No noticeable impact", "1": "Reduced duty but operating", "2": "Major loss of duty or unit unusable"}, "probabilities": {"0": 0.05, "1": 0.67, "2": 0.28}}}</t>
+          <t>{"input_tokens": 487, "output_tokens": 102}</t>
+        </is>
+      </c>
+      <c r="C5" s="35" t="inlineStr">
+        <is>
+          <t>{"hx_problem": {"type": "choice", "choice": "tube_leak", "confidence": 1.0, "probabilities": {"other": 0.0, "flow_maldistribution": 0.0, "tube_leak": 1.0, "control_valve": 0.0, "fouling": 0.0}}, "hx_crosscontam": {"type": "noul", "noul": 0.9}, "hx_impact": {"type": "score", "score": 1.25, "confidence": 0.51, "legend": {"0": "No noticeable impact", "1": "Reduced duty but operating", "2": "Major loss of duty or unit unusable"}, "probabilities": {"0": 0.04, "1": 0.67, "2": 0.29}}}</t>
         </is>
       </c>
     </row>
@@ -16581,7 +16656,12 @@
       </c>
       <c r="B6" s="35" t="inlineStr">
         <is>
-          <t>{"col_symptom": {"type": "choice", "choice": "flooding", "confidence": 0.89, "probabilities": {"instrument": 0.02, "weeping": 0.0, "flooding": 0.91, "fouling": 0.0, "foaming": 0.06, "reboiler_condenser": 0.0, "other": 0.01}}, "col_offspec": {"type": "noul", "noul": 0.99}, "col_stability": {"type": "score", "score": 2.0, "confidence": 1.0, "legend": {"0": "Steady operation", "1": "Drifting or minor swings", "2": "Significant upset"}, "probabilities": {"0": 0.0, "1": 0.0, "2": 1.0}}}</t>
+          <t>{"input_tokens": 514, "output_tokens": 117}</t>
+        </is>
+      </c>
+      <c r="C6" s="35" t="inlineStr">
+        <is>
+          <t>{"col_symptom": {"type": "choice", "choice": "flooding", "confidence": 0.84, "probabilities": {"instrument": 0.02, "flooding": 0.86, "fouling": 0.01, "other": 0.02, "reboiler_condenser": 0.0, "weeping": 0.0, "foaming": 0.09}}, "col_offspec": {"type": "noul", "noul": 0.99}, "col_stability": {"type": "score", "score": 2.0, "confidence": 1.0, "legend": {"0": "Steady operation", "1": "Drifting or minor swings", "2": "Significant upset"}, "probabilities": {"0": 0.0, "1": 0.0, "2": 1.0}}}</t>
         </is>
       </c>
     </row>
@@ -16593,7 +16673,12 @@
       </c>
       <c r="B7" s="35" t="inlineStr">
         <is>
-          <t>{"col_symptom": {"type": "choice", "choice": "other", "confidence": 1.0, "probabilities": {"foaming": 0.0, "reboiler_condenser": 0.0, "fouling": 0.0, "other": 1.0, "instrument": 0.0, "flooding": 0.0, "weeping": 0.0}}, "col_offspec": {"type": "noul", "noul": 0.01}, "col_stability": {"type": "score", "score": 0.0, "confidence": 1.0, "legend": {"0": "Steady operation", "1": "Drifting or minor swings", "2": "Significant upset"}, "probabilities": {"0": 1.0, "1": 0.0, "2": 0.0}}}</t>
+          <t>{"input_tokens": 512, "output_tokens": 115}</t>
+        </is>
+      </c>
+      <c r="C7" s="35" t="inlineStr">
+        <is>
+          <t>{"col_symptom": {"type": "choice", "choice": "other", "confidence": 1.0, "probabilities": {"other": 1.0, "flooding": 0.0, "reboiler_condenser": 0.0, "foaming": 0.0, "instrument": 0.0, "fouling": 0.0, "weeping": 0.0}}, "col_offspec": {"type": "noul", "noul": 0.01}, "col_stability": {"type": "score", "score": 0.0, "confidence": 1.0, "legend": {"0": "Steady operation", "1": "Drifting or minor swings", "2": "Significant upset"}, "probabilities": {"0": 1.0, "1": 0.0, "2": 0.0}}}</t>
         </is>
       </c>
     </row>
@@ -16739,7 +16824,7 @@
         <v>0</v>
       </c>
       <c r="F3" s="35" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.945</v>
       </c>
       <c r="G3" s="35" t="n">
         <v>2</v>
@@ -16751,7 +16836,7 @@
         <v>1</v>
       </c>
       <c r="J3" s="35" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.945</v>
       </c>
       <c r="K3" s="35" t="inlineStr"/>
     </row>
@@ -16776,7 +16861,7 @@
         <v>0</v>
       </c>
       <c r="F4" s="35" t="n">
-        <v>0.985</v>
+        <v>0.99</v>
       </c>
       <c r="G4" s="35" t="n">
         <v>2</v>
@@ -16788,7 +16873,7 @@
         <v>1</v>
       </c>
       <c r="J4" s="35" t="n">
-        <v>0.985</v>
+        <v>0.99</v>
       </c>
       <c r="K4" s="35" t="inlineStr"/>
     </row>
@@ -16850,7 +16935,7 @@
         <v>0</v>
       </c>
       <c r="F6" s="35" t="n">
-        <v>0.89</v>
+        <v>0.885</v>
       </c>
       <c r="G6" s="35" t="n">
         <v>2</v>
@@ -16862,7 +16947,7 @@
         <v>1</v>
       </c>
       <c r="J6" s="35" t="n">
-        <v>0.89</v>
+        <v>0.885</v>
       </c>
       <c r="K6" s="35" t="inlineStr"/>
     </row>
@@ -16887,7 +16972,7 @@
         <v>1</v>
       </c>
       <c r="F7" s="35" t="n">
-        <v>0.66</v>
+        <v>0.675</v>
       </c>
       <c r="G7" s="35" t="n">
         <v>2</v>
@@ -16899,7 +16984,7 @@
         <v>0.5</v>
       </c>
       <c r="J7" s="35" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.84</v>
       </c>
       <c r="K7" s="35" t="n">
         <v>0.51</v>
@@ -16926,7 +17011,7 @@
         <v>0</v>
       </c>
       <c r="F8" s="35" t="n">
-        <v>0.945</v>
+        <v>0.92</v>
       </c>
       <c r="G8" s="35" t="n">
         <v>2</v>
@@ -16938,7 +17023,7 @@
         <v>1</v>
       </c>
       <c r="J8" s="35" t="n">
-        <v>0.945</v>
+        <v>0.92</v>
       </c>
       <c r="K8" s="35" t="inlineStr"/>
     </row>

</xml_diff>